<commit_message>
stop loso_refit dying when there is nothing to rescore
</commit_message>
<xml_diff>
--- a/04_Features/modules/contrast_networks/c_data/contrast_stability.xlsx
+++ b/04_Features/modules/contrast_networks/c_data/contrast_stability.xlsx
@@ -8,12 +8,13 @@
   <sheets>
     <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="module_stability" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="provenance" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t xml:space="preserve">contrast</t>
   </si>
@@ -63,15 +64,27 @@
     <t xml:space="preserve">brown</t>
   </si>
   <si>
+    <t xml:space="preserve">cyan</t>
+  </si>
+  <si>
     <t xml:space="preserve">green</t>
   </si>
   <si>
     <t xml:space="preserve">greenyellow</t>
   </si>
   <si>
+    <t xml:space="preserve">grey60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lightcyan</t>
+  </si>
+  <si>
     <t xml:space="preserve">magenta</t>
   </si>
   <si>
+    <t xml:space="preserve">midnightblue</t>
+  </si>
+  <si>
     <t xml:space="preserve">pink</t>
   </si>
   <si>
@@ -93,19 +106,10 @@
     <t xml:space="preserve">yellow</t>
   </si>
   <si>
-    <t xml:space="preserve">cyan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">grey60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lightcyan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lightgreen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">midnightblue</t>
+    <t xml:space="preserve">fingerprint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4aaa828a692f</t>
   </si>
 </sst>
 </file>
@@ -462,16 +466,16 @@
         <v>14</v>
       </c>
       <c r="C2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D2" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0.365450332866949</v>
+        <v>0.299375072579028</v>
       </c>
     </row>
     <row r="3">
@@ -485,13 +489,13 @@
         <v>12</v>
       </c>
       <c r="D3" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0.351000490367605</v>
+        <v>0.388374607248449</v>
       </c>
     </row>
   </sheetData>
@@ -533,16 +537,16 @@
         <v>13</v>
       </c>
       <c r="C2" t="n">
-        <v>0.365450332866949</v>
+        <v>0.294091038267693</v>
       </c>
       <c r="D2" t="n">
-        <v>0.11340206185567</v>
+        <v>0.0818181818181818</v>
       </c>
       <c r="E2" t="n">
         <v>14</v>
       </c>
       <c r="F2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
@@ -553,16 +557,16 @@
         <v>14</v>
       </c>
       <c r="C3" t="n">
-        <v>0.387458526953199</v>
+        <v>0.408622408705999</v>
       </c>
       <c r="D3" t="n">
-        <v>0.217898832684825</v>
+        <v>0.246710526315789</v>
       </c>
       <c r="E3" t="n">
         <v>14</v>
       </c>
       <c r="F3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -573,16 +577,16 @@
         <v>15</v>
       </c>
       <c r="C4" t="n">
-        <v>0.415854770764466</v>
+        <v>0.62578935471953</v>
       </c>
       <c r="D4" t="n">
-        <v>0.323144104803493</v>
+        <v>0.540540540540541</v>
       </c>
       <c r="E4" t="n">
         <v>14</v>
       </c>
       <c r="F4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -593,16 +597,16 @@
         <v>16</v>
       </c>
       <c r="C5" t="n">
-        <v>0.359206046056766</v>
+        <v>0.300946554415068</v>
       </c>
       <c r="D5" t="n">
-        <v>0.19047619047619</v>
+        <v>0.175</v>
       </c>
       <c r="E5" t="n">
         <v>14</v>
       </c>
       <c r="F5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -613,16 +617,16 @@
         <v>17</v>
       </c>
       <c r="C6" t="n">
-        <v>0.376736949901292</v>
+        <v>0.388877324568445</v>
       </c>
       <c r="D6" t="n">
-        <v>0.065359477124183</v>
+        <v>0.224242424242424</v>
       </c>
       <c r="E6" t="n">
         <v>14</v>
       </c>
       <c r="F6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
@@ -633,10 +637,10 @@
         <v>18</v>
       </c>
       <c r="C7" t="n">
-        <v>0.283553600168952</v>
+        <v>0.219410113815316</v>
       </c>
       <c r="D7" t="n">
-        <v>0.194915254237288</v>
+        <v>0.13265306122449</v>
       </c>
       <c r="E7" t="n">
         <v>14</v>
@@ -653,10 +657,10 @@
         <v>19</v>
       </c>
       <c r="C8" t="n">
-        <v>0.294658442837154</v>
+        <v>0.234775636065655</v>
       </c>
       <c r="D8" t="n">
-        <v>0.186746987951807</v>
+        <v>0.0919540229885057</v>
       </c>
       <c r="E8" t="n">
         <v>14</v>
@@ -673,16 +677,16 @@
         <v>20</v>
       </c>
       <c r="C9" t="n">
-        <v>0.286285582283498</v>
+        <v>0.395036736798871</v>
       </c>
       <c r="D9" t="n">
-        <v>0.159574468085106</v>
+        <v>0.171052631578947</v>
       </c>
       <c r="E9" t="n">
         <v>14</v>
       </c>
       <c r="F9" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -693,16 +697,16 @@
         <v>21</v>
       </c>
       <c r="C10" t="n">
-        <v>0.637563447352626</v>
+        <v>0.322325878872328</v>
       </c>
       <c r="D10" t="n">
-        <v>0.362068965517241</v>
+        <v>0.0578512396694215</v>
       </c>
       <c r="E10" t="n">
         <v>14</v>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11">
@@ -713,16 +717,16 @@
         <v>22</v>
       </c>
       <c r="C11" t="n">
-        <v>0.353971978651961</v>
+        <v>0.294540936835289</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0252100840336134</v>
+        <v>0.136363636363636</v>
       </c>
       <c r="E11" t="n">
         <v>14</v>
       </c>
       <c r="F11" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12">
@@ -733,16 +737,16 @@
         <v>23</v>
       </c>
       <c r="C12" t="n">
-        <v>0.352957789417806</v>
+        <v>0.299375072579028</v>
       </c>
       <c r="D12" t="n">
-        <v>0.107142857142857</v>
+        <v>0.048</v>
       </c>
       <c r="E12" t="n">
         <v>14</v>
       </c>
       <c r="F12" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -753,16 +757,16 @@
         <v>24</v>
       </c>
       <c r="C13" t="n">
-        <v>0.645670491400015</v>
+        <v>0.237159165488933</v>
       </c>
       <c r="D13" t="n">
-        <v>0.387434554973822</v>
+        <v>0.106796116504854</v>
       </c>
       <c r="E13" t="n">
         <v>14</v>
       </c>
       <c r="F13" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
@@ -773,53 +777,53 @@
         <v>25</v>
       </c>
       <c r="C14" t="n">
-        <v>0.383276217156384</v>
+        <v>0.269220065108779</v>
       </c>
       <c r="D14" t="n">
-        <v>0.254416961130742</v>
+        <v>0.1375</v>
       </c>
       <c r="E14" t="n">
         <v>14</v>
       </c>
       <c r="F14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="C15" t="n">
-        <v>0.383163653461182</v>
+        <v>0.264638766901275</v>
       </c>
       <c r="D15" t="n">
-        <v>0.189393939393939</v>
+        <v>0.0448717948717949</v>
       </c>
       <c r="E15" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F15" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="C16" t="n">
-        <v>0.346238356118535</v>
+        <v>0.23791300860068</v>
       </c>
       <c r="D16" t="n">
-        <v>0.246305418719212</v>
+        <v>0.103626943005181</v>
       </c>
       <c r="E16" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F16" t="n">
         <v>14</v>
@@ -827,42 +831,42 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C17" t="n">
-        <v>0.440575723559228</v>
+        <v>0.662135682787544</v>
       </c>
       <c r="D17" t="n">
-        <v>0.269886363636364</v>
+        <v>0.386308068459658</v>
       </c>
       <c r="E17" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F17" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C18" t="n">
-        <v>0.324745658334526</v>
+        <v>0.420117958465615</v>
       </c>
       <c r="D18" t="n">
-        <v>0.137614678899083</v>
+        <v>0.229437229437229</v>
       </c>
       <c r="E18" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F18" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19">
@@ -870,19 +874,19 @@
         <v>7</v>
       </c>
       <c r="B19" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C19" t="n">
-        <v>0.377050617015592</v>
+        <v>0.459148826148781</v>
       </c>
       <c r="D19" t="n">
-        <v>0.148648648648649</v>
+        <v>0.225</v>
       </c>
       <c r="E19" t="n">
         <v>15</v>
       </c>
       <c r="F19" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20">
@@ -890,19 +894,19 @@
         <v>7</v>
       </c>
       <c r="B20" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C20" t="n">
-        <v>0.46041057492111</v>
+        <v>0.319774145094041</v>
       </c>
       <c r="D20" t="n">
-        <v>0.145454545454545</v>
+        <v>0.190217391304348</v>
       </c>
       <c r="E20" t="n">
         <v>15</v>
       </c>
       <c r="F20" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21">
@@ -910,13 +914,13 @@
         <v>7</v>
       </c>
       <c r="B21" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C21" t="n">
-        <v>0.213356992878642</v>
+        <v>0.402471413385647</v>
       </c>
       <c r="D21" t="n">
-        <v>0.050314465408805</v>
+        <v>0.266409266409266</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -930,13 +934,13 @@
         <v>7</v>
       </c>
       <c r="B22" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="C22" t="n">
-        <v>0.205889059610581</v>
+        <v>0.337070092246932</v>
       </c>
       <c r="D22" t="n">
-        <v>0.036144578313253</v>
+        <v>0.15</v>
       </c>
       <c r="E22" t="n">
         <v>15</v>
@@ -950,19 +954,19 @@
         <v>7</v>
       </c>
       <c r="B23" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C23" t="n">
-        <v>0.122045005982097</v>
+        <v>0.395521875999874</v>
       </c>
       <c r="D23" t="n">
-        <v>0.0619469026548673</v>
+        <v>0.186170212765957</v>
       </c>
       <c r="E23" t="n">
         <v>15</v>
       </c>
       <c r="F23" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24">
@@ -973,16 +977,16 @@
         <v>18</v>
       </c>
       <c r="C24" t="n">
-        <v>0.419824302497543</v>
+        <v>0.441450846275417</v>
       </c>
       <c r="D24" t="n">
-        <v>0.253623188405797</v>
+        <v>0.126126126126126</v>
       </c>
       <c r="E24" t="n">
         <v>15</v>
       </c>
       <c r="F24" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25">
@@ -990,19 +994,19 @@
         <v>7</v>
       </c>
       <c r="B25" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C25" t="n">
-        <v>0.34866097194778</v>
+        <v>0.19098446054779</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0935251798561151</v>
+        <v>0.101123595505618</v>
       </c>
       <c r="E25" t="n">
         <v>15</v>
       </c>
       <c r="F25" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26">
@@ -1010,19 +1014,19 @@
         <v>7</v>
       </c>
       <c r="B26" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C26" t="n">
-        <v>0.512084025078659</v>
+        <v>0.523122912417499</v>
       </c>
       <c r="D26" t="n">
-        <v>0.385416666666667</v>
+        <v>0.27906976744186</v>
       </c>
       <c r="E26" t="n">
         <v>15</v>
       </c>
       <c r="F26" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
@@ -1030,19 +1034,19 @@
         <v>7</v>
       </c>
       <c r="B27" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C27" t="n">
-        <v>0.352448309523242</v>
+        <v>0.197163039554047</v>
       </c>
       <c r="D27" t="n">
-        <v>0.153333333333333</v>
+        <v>0.053030303030303</v>
       </c>
       <c r="E27" t="n">
         <v>15</v>
       </c>
       <c r="F27" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28">
@@ -1050,13 +1054,13 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C28" t="n">
-        <v>0.402602343742542</v>
+        <v>0.296903707809413</v>
       </c>
       <c r="D28" t="n">
-        <v>0.214876033057851</v>
+        <v>0.0666666666666667</v>
       </c>
       <c r="E28" t="n">
         <v>15</v>
@@ -1070,19 +1074,19 @@
         <v>7</v>
       </c>
       <c r="B29" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C29" t="n">
-        <v>0.349552671211968</v>
+        <v>0.34819142192053</v>
       </c>
       <c r="D29" t="n">
-        <v>0.018018018018018</v>
+        <v>0.152671755725191</v>
       </c>
       <c r="E29" t="n">
         <v>15</v>
       </c>
       <c r="F29" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="30">
@@ -1090,19 +1094,19 @@
         <v>7</v>
       </c>
       <c r="B30" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C30" t="n">
-        <v>0.30916499701151</v>
+        <v>0.290997787478457</v>
       </c>
       <c r="D30" t="n">
-        <v>0.175</v>
+        <v>0.0584415584415584</v>
       </c>
       <c r="E30" t="n">
         <v>15</v>
       </c>
       <c r="F30" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="31">
@@ -1110,19 +1114,19 @@
         <v>7</v>
       </c>
       <c r="B31" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C31" t="n">
-        <v>0.771505175421908</v>
+        <v>0.381227338497023</v>
       </c>
       <c r="D31" t="n">
-        <v>0.648648648648649</v>
+        <v>0.236220472440945</v>
       </c>
       <c r="E31" t="n">
         <v>15</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32">
@@ -1130,19 +1134,80 @@
         <v>7</v>
       </c>
       <c r="B32" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C32" t="n">
-        <v>0.301000671251151</v>
+        <v>0.401496588388175</v>
       </c>
       <c r="D32" t="n">
-        <v>0.181286549707602</v>
+        <v>0.210084033613445</v>
       </c>
       <c r="E32" t="n">
         <v>15</v>
       </c>
       <c r="F32" t="n">
-        <v>14</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>7</v>
+      </c>
+      <c r="B33" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.761610091703527</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.642441860465116</v>
+      </c>
+      <c r="E33" t="n">
+        <v>15</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>7</v>
+      </c>
+      <c r="B34" t="s">
+        <v>29</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.453760567676295</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.20817843866171</v>
+      </c>
+      <c r="E34" t="n">
+        <v>15</v>
+      </c>
+      <c r="F34" t="n">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>